<commit_message>
Update notice.xlsx from SARC website admin
</commit_message>
<xml_diff>
--- a/notice.xlsx
+++ b/notice.xlsx
@@ -461,7 +461,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -478,9 +478,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>